<commit_message>
Eliminar archivos .tex del repositorio y agregar a .gitignore
Los archivos LaTeX de la tesis se gestionan localmente (Overleaf/local).
Se actualiza resultados_semana.xlsx con registro del 2026-04-05.
</commit_message>
<xml_diff>
--- a/resultados_semana.xlsx
+++ b/resultados_semana.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X55"/>
+  <dimension ref="A1:X67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4088,9 +4088,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V38" t="inlineStr"/>
-      <c r="W38" t="inlineStr"/>
-      <c r="X38" t="inlineStr"/>
+      <c r="V38" t="n">
+        <v>246.630005</v>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4174,9 +4184,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr"/>
-      <c r="X39" t="inlineStr"/>
+      <c r="V39" t="n">
+        <v>200.949997</v>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4260,9 +4280,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V40" t="inlineStr"/>
-      <c r="W40" t="inlineStr"/>
-      <c r="X40" t="inlineStr"/>
+      <c r="V40" t="n">
+        <v>273.5</v>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4346,9 +4376,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V41" t="inlineStr"/>
-      <c r="W41" t="inlineStr"/>
-      <c r="X41" t="inlineStr"/>
+      <c r="V41" t="n">
+        <v>536.380005</v>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4432,9 +4472,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V42" t="inlineStr"/>
-      <c r="W42" t="inlineStr"/>
-      <c r="X42" t="inlineStr"/>
+      <c r="V42" t="n">
+        <v>358.959991</v>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4518,9 +4568,19 @@
           <t>Riesgo ALTO: Esta inversión es arriesgada. Solo invierte dinero que puedas perder.</t>
         </is>
       </c>
-      <c r="V43" t="inlineStr"/>
-      <c r="W43" t="inlineStr"/>
-      <c r="X43" t="inlineStr"/>
+      <c r="V43" t="n">
+        <v>355.279999</v>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4604,9 +4664,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V44" t="inlineStr"/>
-      <c r="W44" t="inlineStr"/>
-      <c r="X44" t="inlineStr"/>
+      <c r="V44" t="n">
+        <v>253.789993</v>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>SUBIDA</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4690,9 +4760,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V45" t="inlineStr"/>
-      <c r="W45" t="inlineStr"/>
-      <c r="X45" t="inlineStr"/>
+      <c r="V45" t="n">
+        <v>208.270004</v>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>SUBIDA</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4776,9 +4856,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr"/>
-      <c r="W46" t="inlineStr"/>
-      <c r="X46" t="inlineStr"/>
+      <c r="V46" t="n">
+        <v>287.559998</v>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>SUBIDA</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4862,9 +4952,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V47" t="inlineStr"/>
-      <c r="W47" t="inlineStr"/>
-      <c r="X47" t="inlineStr"/>
+      <c r="V47" t="n">
+        <v>572.130005</v>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>SUBIDA</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4948,9 +5048,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V48" t="inlineStr"/>
-      <c r="W48" t="inlineStr"/>
-      <c r="X48" t="inlineStr"/>
+      <c r="V48" t="n">
+        <v>370.170013</v>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>SUBIDA</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5034,9 +5144,19 @@
           <t>Riesgo ALTO: Esta inversión es arriesgada. Solo invierte dinero que puedas perder.</t>
         </is>
       </c>
-      <c r="V49" t="inlineStr"/>
-      <c r="W49" t="inlineStr"/>
-      <c r="X49" t="inlineStr"/>
+      <c r="V49" t="n">
+        <v>371.75</v>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>SUBIDA</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5120,9 +5240,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V50" t="inlineStr"/>
-      <c r="W50" t="inlineStr"/>
-      <c r="X50" t="inlineStr"/>
+      <c r="V50" t="n">
+        <v>255.919998</v>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>SUBIDA</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5206,9 +5336,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V51" t="inlineStr"/>
-      <c r="W51" t="inlineStr"/>
-      <c r="X51" t="inlineStr"/>
+      <c r="V51" t="n">
+        <v>209.770004</v>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>SUBIDA</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5292,9 +5432,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V52" t="inlineStr"/>
-      <c r="W52" t="inlineStr"/>
-      <c r="X52" t="inlineStr"/>
+      <c r="V52" t="n">
+        <v>295.769989</v>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>SUBIDA</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5378,9 +5528,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V53" t="inlineStr"/>
-      <c r="W53" t="inlineStr"/>
-      <c r="X53" t="inlineStr"/>
+      <c r="V53" t="n">
+        <v>574.460022</v>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>SUBIDA</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5464,9 +5624,19 @@
           <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
         </is>
       </c>
-      <c r="V54" t="inlineStr"/>
-      <c r="W54" t="inlineStr"/>
-      <c r="X54" t="inlineStr"/>
+      <c r="V54" t="n">
+        <v>373.459991</v>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>SUBIDA</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5550,9 +5720,1051 @@
           <t>Riesgo ALTO: Esta inversión es arriesgada. Solo invierte dinero que puedas perder.</t>
         </is>
       </c>
-      <c r="V55" t="inlineStr"/>
-      <c r="W55" t="inlineStr"/>
-      <c r="X55" t="inlineStr"/>
+      <c r="V55" t="n">
+        <v>360.589996</v>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>SUBIDA</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>18:18:37</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>255.9199981689453</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0.1134</v>
+      </c>
+      <c r="F56" t="n">
+        <v>253.4105</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>252.1179</v>
+      </c>
+      <c r="I56" t="n">
+        <v>-1.4857</v>
+      </c>
+      <c r="J56" t="n">
+        <v>3</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="M56" t="n">
+        <v>0.5891891891891892</v>
+      </c>
+      <c r="N56" t="n">
+        <v>0.6078205128205127</v>
+      </c>
+      <c r="O56" t="n">
+        <v>0.3657705834176422</v>
+      </c>
+      <c r="P56" t="n">
+        <v>0.3783687730263073</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>0.5563207123874852</v>
+      </c>
+      <c r="R56" t="n">
+        <v>0.3935</v>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>venta</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="inlineStr"/>
+      <c r="X56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>18:19:05</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>209.7700042724609</v>
+      </c>
+      <c r="E57" t="n">
+        <v>-0.3799</v>
+      </c>
+      <c r="F57" t="n">
+        <v>209.3675</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
+        <v>206.8268</v>
+      </c>
+      <c r="I57" t="n">
+        <v>-1.4031</v>
+      </c>
+      <c r="J57" t="n">
+        <v>3</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>gradient_boosting</t>
+        </is>
+      </c>
+      <c r="M57" t="n">
+        <v>0.5216216216216216</v>
+      </c>
+      <c r="N57" t="n">
+        <v>0.4610472472741957</v>
+      </c>
+      <c r="O57" t="n">
+        <v>0.340112443778111</v>
+      </c>
+      <c r="P57" t="n">
+        <v>0.3673507312980998</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>0.5634585447917753</v>
+      </c>
+      <c r="R57" t="n">
+        <v>0.0641</v>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>venta</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr"/>
+      <c r="W57" t="inlineStr"/>
+      <c r="X57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>18:18:46</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>295.7699890136719</v>
+      </c>
+      <c r="E58" t="n">
+        <v>-0.5447</v>
+      </c>
+      <c r="F58" t="n">
+        <v>297.5725</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>290.7346</v>
+      </c>
+      <c r="I58" t="n">
+        <v>-1.7025</v>
+      </c>
+      <c r="J58" t="n">
+        <v>3</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="M58" t="n">
+        <v>0.5108108108108109</v>
+      </c>
+      <c r="N58" t="n">
+        <v>0.5843588620023695</v>
+      </c>
+      <c r="O58" t="n">
+        <v>0.5244576719576719</v>
+      </c>
+      <c r="P58" t="n">
+        <v>0.485265279105109</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>0.6046503187547758</v>
+      </c>
+      <c r="R58" t="n">
+        <v>-0.0902</v>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>venta</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr"/>
+      <c r="W58" t="inlineStr"/>
+      <c r="X58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>18:19:24</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>574.4600219726562</v>
+      </c>
+      <c r="E59" t="n">
+        <v>-0.8235</v>
+      </c>
+      <c r="F59" t="n">
+        <v>602.1627</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>bajista</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>563.9355</v>
+      </c>
+      <c r="I59" t="n">
+        <v>-1.8321</v>
+      </c>
+      <c r="J59" t="n">
+        <v>3</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="M59" t="n">
+        <v>0.5232876712328768</v>
+      </c>
+      <c r="N59" t="n">
+        <v>0.4449544817927171</v>
+      </c>
+      <c r="O59" t="n">
+        <v>0.5172315778806651</v>
+      </c>
+      <c r="P59" t="n">
+        <v>0.4188848653019456</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>0.5129436534507528</v>
+      </c>
+      <c r="R59" t="n">
+        <v>0.0442</v>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>venta</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr"/>
+      <c r="W59" t="inlineStr"/>
+      <c r="X59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>18:18:56</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>373.4599914550781</v>
+      </c>
+      <c r="E60" t="n">
+        <v>1.1073</v>
+      </c>
+      <c r="F60" t="n">
+        <v>385.497</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>bajista</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>369.1343</v>
+      </c>
+      <c r="I60" t="n">
+        <v>-1.1583</v>
+      </c>
+      <c r="J60" t="n">
+        <v>3</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>gradient_boosting</t>
+        </is>
+      </c>
+      <c r="M60" t="n">
+        <v>0.5216216216216216</v>
+      </c>
+      <c r="N60" t="n">
+        <v>0.515767575322812</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0.4550648032762662</v>
+      </c>
+      <c r="P60" t="n">
+        <v>0.3937281264351434</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>0.5900000253946202</v>
+      </c>
+      <c r="R60" t="n">
+        <v>0.204</v>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>venta</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr"/>
+      <c r="W60" t="inlineStr"/>
+      <c r="X60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>18:19:15</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>360.5899963378906</v>
+      </c>
+      <c r="E61" t="n">
+        <v>-5.4215</v>
+      </c>
+      <c r="F61" t="n">
+        <v>383.86</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="H61" t="n">
+        <v>347.7785</v>
+      </c>
+      <c r="I61" t="n">
+        <v>-3.5529</v>
+      </c>
+      <c r="J61" t="n">
+        <v>3</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>gradient_boosting</t>
+        </is>
+      </c>
+      <c r="M61" t="n">
+        <v>0.5108108108108109</v>
+      </c>
+      <c r="N61" t="n">
+        <v>0.4754091110128262</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0.3929264828738513</v>
+      </c>
+      <c r="P61" t="n">
+        <v>0.397265236670271</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>0.5386603510614916</v>
+      </c>
+      <c r="R61" t="n">
+        <v>-0.0408</v>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>venta</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>Riesgo ALTO: Esta inversión es arriesgada. Solo invierte dinero que puedas perder.</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr"/>
+      <c r="W61" t="inlineStr"/>
+      <c r="X61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>18:58:18</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>255.9199981689453</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.1134</v>
+      </c>
+      <c r="F62" t="n">
+        <v>253.4105</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="H62" t="n">
+        <v>252.1198</v>
+      </c>
+      <c r="I62" t="n">
+        <v>-1.4849</v>
+      </c>
+      <c r="J62" t="n">
+        <v>3</v>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="M62" t="n">
+        <v>0.5891891891891892</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0.6078205128205127</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0.3657705834176422</v>
+      </c>
+      <c r="P62" t="n">
+        <v>0.3783687730263073</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>0.5548305163090537</v>
+      </c>
+      <c r="R62" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>venta</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr"/>
+      <c r="W62" t="inlineStr"/>
+      <c r="X62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>18:58:47</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>209.7700042724609</v>
+      </c>
+      <c r="E63" t="n">
+        <v>-0.3799</v>
+      </c>
+      <c r="F63" t="n">
+        <v>209.3675</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>206.8268</v>
+      </c>
+      <c r="I63" t="n">
+        <v>-1.4031</v>
+      </c>
+      <c r="J63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>gradient_boosting</t>
+        </is>
+      </c>
+      <c r="M63" t="n">
+        <v>0.5216216216216216</v>
+      </c>
+      <c r="N63" t="n">
+        <v>0.4610472472741957</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0.340112443778111</v>
+      </c>
+      <c r="P63" t="n">
+        <v>0.3673507312980998</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>0.5634585447917753</v>
+      </c>
+      <c r="R63" t="n">
+        <v>0.2685</v>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>venta</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr"/>
+      <c r="W63" t="inlineStr"/>
+      <c r="X63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>18:58:28</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>295.7699890136719</v>
+      </c>
+      <c r="E64" t="n">
+        <v>-0.5447</v>
+      </c>
+      <c r="F64" t="n">
+        <v>297.5725</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="H64" t="n">
+        <v>290.7338</v>
+      </c>
+      <c r="I64" t="n">
+        <v>-1.7027</v>
+      </c>
+      <c r="J64" t="n">
+        <v>3</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="M64" t="n">
+        <v>0.5135135135135135</v>
+      </c>
+      <c r="N64" t="n">
+        <v>0.5773781291172595</v>
+      </c>
+      <c r="O64" t="n">
+        <v>0.5262037037037037</v>
+      </c>
+      <c r="P64" t="n">
+        <v>0.4907718150528214</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>0.6082015193449568</v>
+      </c>
+      <c r="R64" t="n">
+        <v>-0.3336</v>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>negativo</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>venta</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr"/>
+      <c r="W64" t="inlineStr"/>
+      <c r="X64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>18:59:07</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>574.4600219726562</v>
+      </c>
+      <c r="E65" t="n">
+        <v>-0.8235</v>
+      </c>
+      <c r="F65" t="n">
+        <v>602.1627</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>bajista</t>
+        </is>
+      </c>
+      <c r="H65" t="n">
+        <v>564.1653</v>
+      </c>
+      <c r="I65" t="n">
+        <v>-1.7921</v>
+      </c>
+      <c r="J65" t="n">
+        <v>3</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="M65" t="n">
+        <v>0.5342465753424657</v>
+      </c>
+      <c r="N65" t="n">
+        <v>0.4562160025300442</v>
+      </c>
+      <c r="O65" t="n">
+        <v>0.524128129604803</v>
+      </c>
+      <c r="P65" t="n">
+        <v>0.4284250813440428</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>0.5090724401474909</v>
+      </c>
+      <c r="R65" t="n">
+        <v>0.0697</v>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>venta</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr"/>
+      <c r="W65" t="inlineStr"/>
+      <c r="X65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>18:58:38</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>373.4599914550781</v>
+      </c>
+      <c r="E66" t="n">
+        <v>1.1073</v>
+      </c>
+      <c r="F66" t="n">
+        <v>385.497</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>bajista</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
+        <v>369.2846</v>
+      </c>
+      <c r="I66" t="n">
+        <v>-1.118</v>
+      </c>
+      <c r="J66" t="n">
+        <v>3</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>gradient_boosting</t>
+        </is>
+      </c>
+      <c r="M66" t="n">
+        <v>0.5108108108108109</v>
+      </c>
+      <c r="N66" t="n">
+        <v>0.5101307189542483</v>
+      </c>
+      <c r="O66" t="n">
+        <v>0.4550648032762662</v>
+      </c>
+      <c r="P66" t="n">
+        <v>0.3886450374810867</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>0.5885624692400828</v>
+      </c>
+      <c r="R66" t="n">
+        <v>0.1615</v>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>venta</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>Riesgo MODERADO: Riesgo normal de mercado. Podrías ganar o perder.</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr"/>
+      <c r="W66" t="inlineStr"/>
+      <c r="X66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>18:58:57</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>360.5899963378906</v>
+      </c>
+      <c r="E67" t="n">
+        <v>-5.4215</v>
+      </c>
+      <c r="F67" t="n">
+        <v>383.86</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="H67" t="n">
+        <v>347.7785</v>
+      </c>
+      <c r="I67" t="n">
+        <v>-3.5529</v>
+      </c>
+      <c r="J67" t="n">
+        <v>3</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>BAJADA</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>gradient_boosting</t>
+        </is>
+      </c>
+      <c r="M67" t="n">
+        <v>0.5108108108108109</v>
+      </c>
+      <c r="N67" t="n">
+        <v>0.4754091110128262</v>
+      </c>
+      <c r="O67" t="n">
+        <v>0.3929264828738513</v>
+      </c>
+      <c r="P67" t="n">
+        <v>0.397265236670271</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>0.5386603510614916</v>
+      </c>
+      <c r="R67" t="n">
+        <v>-0.1265</v>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>negativo</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>venta</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>Riesgo ALTO: Esta inversión es arriesgada. Solo invierte dinero que puedas perder.</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr"/>
+      <c r="W67" t="inlineStr"/>
+      <c r="X67" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>